<commit_message>
Docs: tracker with IPO-number sheet + NHS background-IP contract clause draft
</commit_message>
<xml_diff>
--- a/docs/security/AEGIS-COMPLIANCE-TRACKER.xlsx
+++ b/docs/security/AEGIS-COMPLIANCE-TRACKER.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="Compliance Tracker" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Costs" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Trademarks" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -31,7 +32,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -58,6 +59,11 @@
         <fgColor rgb="00D1E7DD"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004A235A"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -71,12 +77,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1466,4 +1473,240 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="46" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Mark</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>Classes</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>Application № (IPO)</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>Filing date</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>Fee £</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="inlineStr">
+        <is>
+          <t>Payment ref</t>
+        </is>
+      </c>
+      <c r="I1" s="5" t="inlineStr">
+        <is>
+          <t>Renewal due (yr 10)</t>
+        </is>
+      </c>
+      <c r="J1" s="5" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>ZEUS</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Word</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>9, 36, 42, 44, 45</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>NOT FILED - file first</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>445</v>
+      </c>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>File e-TM3; rights from filing date</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>ZEUSTA</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Word</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>9, 36, 42, 44, 45</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>NOT FILED - file first</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>445</v>
+      </c>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Separate application (not a series with ZEUS)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>ZEUS / ZEUS AI / ZEUSAI</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Series (3 marks)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>9, 36, 42, 44, 45</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>NOT FILED - file first</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>505</v>
+      </c>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Series app £205 + 4x£60 classes + £60 extra mark</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>AEGIS</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Word</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>9, 36, 42, 44, 45</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>NOT FILED - file first</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>445</v>
+      </c>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Considered separately per contract timing</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr"/>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" s="3" t="inlineStr"/>
+      <c r="G6" t="n">
+        <v>1840</v>
+      </c>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Series route covers ZEUS+AI variants</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Docs: tracker IPO-number sheet + NHS IP clause draft (PR #28)
* Docs: AEGIS security fixes changelog + operating costs + cost forecast spreadsheet

* Docs: Monday NHS readiness summary

* Docs: trademark applications draft + DTAC submission answers + compliance tracker

* Docs: series application checklist + compliance tracker template + NHS trademark/IP research

* Docs: tracker with IPO-number sheet + NHS background-IP contract clause draft

---------

Co-authored-by: Higgsfield Agent <agent@higgsfield.ai>
</commit_message>
<xml_diff>
--- a/docs/security/AEGIS-COMPLIANCE-TRACKER.xlsx
+++ b/docs/security/AEGIS-COMPLIANCE-TRACKER.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="Compliance Tracker" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Costs" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Trademarks" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -31,7 +32,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -58,6 +59,11 @@
         <fgColor rgb="00D1E7DD"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004A235A"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -71,12 +77,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1466,4 +1473,240 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="46" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Mark</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>Classes</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>Application № (IPO)</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>Filing date</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>Fee £</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="inlineStr">
+        <is>
+          <t>Payment ref</t>
+        </is>
+      </c>
+      <c r="I1" s="5" t="inlineStr">
+        <is>
+          <t>Renewal due (yr 10)</t>
+        </is>
+      </c>
+      <c r="J1" s="5" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>ZEUS</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Word</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>9, 36, 42, 44, 45</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>NOT FILED - file first</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>445</v>
+      </c>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>File e-TM3; rights from filing date</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>ZEUSTA</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Word</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>9, 36, 42, 44, 45</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>NOT FILED - file first</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>445</v>
+      </c>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Separate application (not a series with ZEUS)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>ZEUS / ZEUS AI / ZEUSAI</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Series (3 marks)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>9, 36, 42, 44, 45</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>NOT FILED - file first</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>505</v>
+      </c>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Series app £205 + 4x£60 classes + £60 extra mark</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>AEGIS</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Word</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>9, 36, 42, 44, 45</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>NOT FILED - file first</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>445</v>
+      </c>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Considered separately per contract timing</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr"/>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" s="3" t="inlineStr"/>
+      <c r="G6" t="n">
+        <v>1840</v>
+      </c>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Series route covers ZEUS+AI variants</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>